<commit_message>
Setup for final task in module
</commit_message>
<xml_diff>
--- a/GUNEU_Критерии_оценки_модульной_работы.xlsx
+++ b/GUNEU_Критерии_оценки_модульной_работы.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Учеба\GameDev\Курс Разработчик Unity3d Netologia\GUN38\TankPrototype GUN38\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25465D68-87B2-4E61-BD3C-B07F96D9C92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5F0E51-1851-433A-B928-1981DE252361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="244">
   <si>
     <t>Пункт</t>
   </si>
@@ -802,6 +802,9 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
@@ -1430,21 +1433,12 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1458,7 +1452,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1467,24 +1486,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1739,7 +1742,7 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="14.42578125" customWidth="1"/>
     <col min="6" max="6" width="53.28515625" customWidth="1"/>
-    <col min="7" max="7" width="36.7109375" style="65" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.7109375" style="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="46.5" customHeight="1">
@@ -1761,30 +1764,30 @@
       <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="64" t="s">
+      <c r="G1" s="36" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="12.75">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="55"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="63"/>
       <c r="E2" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.5">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:7" ht="25.5">
       <c r="A4" s="5" t="s">
@@ -1793,13 +1796,13 @@
       <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
       <c r="F4" s="7"/>
-      <c r="G4" s="65" t="s">
+      <c r="G4" s="37" t="s">
         <v>242</v>
       </c>
     </row>
@@ -1810,22 +1813,22 @@
       <c r="B5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="G5" s="65" t="s">
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="G5" s="37" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16.5">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="44"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:7" ht="38.25">
       <c r="A7" s="5" t="s">
@@ -1834,13 +1837,13 @@
       <c r="B7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
       <c r="F7" s="7"/>
-      <c r="G7" s="65" t="s">
+      <c r="G7" s="37" t="s">
         <v>242</v>
       </c>
     </row>
@@ -1851,30 +1854,30 @@
       <c r="B8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
-      <c r="G8" s="65" t="s">
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="G8" s="37" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="12.75">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="47"/>
-      <c r="G9" s="65" t="s">
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="G9" s="37" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="12.75">
-      <c r="A10" s="40"/>
-      <c r="B10" s="41"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="45"/>
       <c r="C10" s="11" t="s">
         <v>19</v>
       </c>
@@ -1885,10 +1888,13 @@
         <v>50</v>
       </c>
       <c r="F10" s="11"/>
+      <c r="G10" s="37" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="12.75">
-      <c r="A11" s="37"/>
-      <c r="B11" s="39"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="46"/>
       <c r="C11" s="14" t="s">
         <v>20</v>
       </c>
@@ -1899,22 +1905,25 @@
         <v>50</v>
       </c>
       <c r="F11" s="14"/>
+      <c r="G11" s="37" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="16.5">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="56"/>
     </row>
     <row r="13" spans="1:7" ht="12.75">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="53" t="s">
         <v>22</v>
       </c>
       <c r="C13" s="11" t="s">
@@ -1927,10 +1936,13 @@
         <v>15</v>
       </c>
       <c r="F13" s="11"/>
+      <c r="G13" s="37" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="12.75">
-      <c r="A14" s="37"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="52"/>
+      <c r="B14" s="46"/>
       <c r="C14" s="11" t="s">
         <v>24</v>
       </c>
@@ -1941,6 +1953,9 @@
         <v>3</v>
       </c>
       <c r="F14" s="11"/>
+      <c r="G14" s="37" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="38.25">
       <c r="A15" s="5" t="s">
@@ -1959,12 +1974,15 @@
         <v>15</v>
       </c>
       <c r="F15" s="11"/>
+      <c r="G15" s="37" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="12.75">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="57" t="s">
+      <c r="B16" s="60" t="s">
         <v>28</v>
       </c>
       <c r="C16" s="11" t="s">
@@ -1977,10 +1995,13 @@
         <v>1</v>
       </c>
       <c r="F16" s="11"/>
-    </row>
-    <row r="17" spans="1:6" ht="12.75">
-      <c r="A17" s="40"/>
-      <c r="B17" s="41"/>
+      <c r="G16" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12.75">
+      <c r="A17" s="51"/>
+      <c r="B17" s="45"/>
       <c r="C17" s="11" t="s">
         <v>30</v>
       </c>
@@ -1991,10 +2012,13 @@
         <v>1</v>
       </c>
       <c r="F17" s="11"/>
-    </row>
-    <row r="18" spans="1:6" ht="12.75">
-      <c r="A18" s="37"/>
-      <c r="B18" s="39"/>
+      <c r="G17" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="12.75">
+      <c r="A18" s="52"/>
+      <c r="B18" s="46"/>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
@@ -2005,12 +2029,15 @@
         <v>5</v>
       </c>
       <c r="F18" s="11"/>
-    </row>
-    <row r="19" spans="1:6" ht="12.75">
-      <c r="A19" s="36" t="s">
+      <c r="G18" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="12.75">
+      <c r="A19" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="60" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="11" t="s">
@@ -2023,10 +2050,13 @@
         <v>10</v>
       </c>
       <c r="F19" s="11"/>
-    </row>
-    <row r="20" spans="1:6" ht="12.75">
-      <c r="A20" s="37"/>
-      <c r="B20" s="39"/>
+      <c r="G19" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="12.75">
+      <c r="A20" s="52"/>
+      <c r="B20" s="46"/>
       <c r="C20" s="11" t="s">
         <v>35</v>
       </c>
@@ -2037,12 +2067,15 @@
         <v>3</v>
       </c>
       <c r="F20" s="11"/>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A21" s="36" t="s">
+      <c r="G20" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A21" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="60" t="s">
         <v>37</v>
       </c>
       <c r="C21" s="11" t="s">
@@ -2055,10 +2088,13 @@
         <v>5</v>
       </c>
       <c r="F21" s="11"/>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A22" s="40"/>
-      <c r="B22" s="41"/>
+      <c r="G21" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A22" s="51"/>
+      <c r="B22" s="45"/>
       <c r="C22" s="11" t="s">
         <v>39</v>
       </c>
@@ -2069,10 +2105,13 @@
         <v>3</v>
       </c>
       <c r="F22" s="11"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="37"/>
-      <c r="B23" s="39"/>
+      <c r="G22" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A23" s="52"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="11" t="s">
         <v>40</v>
       </c>
@@ -2083,12 +2122,15 @@
         <v>5</v>
       </c>
       <c r="F23" s="11"/>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A24" s="36" t="s">
+      <c r="G23" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A24" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="53" t="s">
         <v>42</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -2101,10 +2143,13 @@
         <v>5</v>
       </c>
       <c r="F24" s="11"/>
-    </row>
-    <row r="25" spans="1:6" ht="26.25" customHeight="1">
-      <c r="A25" s="37"/>
-      <c r="B25" s="39"/>
+      <c r="G24" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="26.25" customHeight="1">
+      <c r="A25" s="52"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="11" t="s">
         <v>44</v>
       </c>
@@ -2115,8 +2160,11 @@
         <v>1</v>
       </c>
       <c r="F25" s="11"/>
-    </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G25" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" customHeight="1">
       <c r="A26" s="5" t="s">
         <v>17</v>
       </c>
@@ -2133,12 +2181,15 @@
         <v>10</v>
       </c>
       <c r="F26" s="11"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A27" s="36" t="s">
+      <c r="G26" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A27" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="38" t="s">
+      <c r="B27" s="53" t="s">
         <v>48</v>
       </c>
       <c r="C27" s="11" t="s">
@@ -2151,10 +2202,13 @@
         <v>1</v>
       </c>
       <c r="F27" s="11"/>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A28" s="37"/>
-      <c r="B28" s="39"/>
+      <c r="G27" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A28" s="52"/>
+      <c r="B28" s="46"/>
       <c r="C28" s="11" t="s">
         <v>50</v>
       </c>
@@ -2165,12 +2219,15 @@
         <v>2</v>
       </c>
       <c r="F28" s="11"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A29" s="36" t="s">
+      <c r="G28" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A29" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="B29" s="38" t="s">
+      <c r="B29" s="53" t="s">
         <v>52</v>
       </c>
       <c r="C29" s="11" t="s">
@@ -2183,10 +2240,13 @@
         <v>1</v>
       </c>
       <c r="F29" s="11"/>
-    </row>
-    <row r="30" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A30" s="37"/>
-      <c r="B30" s="39"/>
+      <c r="G29" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="25.5" customHeight="1">
+      <c r="A30" s="52"/>
+      <c r="B30" s="46"/>
       <c r="C30" s="11" t="s">
         <v>54</v>
       </c>
@@ -2197,12 +2257,15 @@
         <v>5</v>
       </c>
       <c r="F30" s="11"/>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A31" s="36" t="s">
+      <c r="G30" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A31" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="58" t="s">
+      <c r="B31" s="57" t="s">
         <v>56</v>
       </c>
       <c r="C31" s="11" t="s">
@@ -2215,10 +2278,13 @@
         <v>1</v>
       </c>
       <c r="F31" s="11"/>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A32" s="40"/>
-      <c r="B32" s="59"/>
+      <c r="G31" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A32" s="51"/>
+      <c r="B32" s="58"/>
       <c r="C32" s="11" t="s">
         <v>58</v>
       </c>
@@ -2229,10 +2295,13 @@
         <v>1</v>
       </c>
       <c r="F32" s="11"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A33" s="40"/>
-      <c r="B33" s="59"/>
+      <c r="G32" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A33" s="51"/>
+      <c r="B33" s="58"/>
       <c r="C33" s="11" t="s">
         <v>59</v>
       </c>
@@ -2243,10 +2312,13 @@
         <v>2</v>
       </c>
       <c r="F33" s="11"/>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A34" s="37"/>
-      <c r="B34" s="60"/>
+      <c r="G33" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A34" s="52"/>
+      <c r="B34" s="59"/>
       <c r="C34" s="11" t="s">
         <v>60</v>
       </c>
@@ -2257,12 +2329,15 @@
         <v>2</v>
       </c>
       <c r="F34" s="11"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A35" s="36" t="s">
+      <c r="G34" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A35" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="53" t="s">
         <v>62</v>
       </c>
       <c r="C35" s="11" t="s">
@@ -2275,10 +2350,13 @@
         <v>2</v>
       </c>
       <c r="F35" s="11"/>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A36" s="40"/>
-      <c r="B36" s="41"/>
+      <c r="G35" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A36" s="51"/>
+      <c r="B36" s="45"/>
       <c r="C36" s="11" t="s">
         <v>64</v>
       </c>
@@ -2289,10 +2367,13 @@
         <v>2</v>
       </c>
       <c r="F36" s="11"/>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A37" s="40"/>
-      <c r="B37" s="41"/>
+      <c r="G36" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A37" s="51"/>
+      <c r="B37" s="45"/>
       <c r="C37" s="11" t="s">
         <v>65</v>
       </c>
@@ -2303,10 +2384,13 @@
         <v>2</v>
       </c>
       <c r="F37" s="11"/>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A38" s="40"/>
-      <c r="B38" s="41"/>
+      <c r="G37" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A38" s="51"/>
+      <c r="B38" s="45"/>
       <c r="C38" s="11" t="s">
         <v>66</v>
       </c>
@@ -2317,10 +2401,13 @@
         <v>4</v>
       </c>
       <c r="F38" s="11"/>
-    </row>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A39" s="40"/>
-      <c r="B39" s="41"/>
+      <c r="G38" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A39" s="51"/>
+      <c r="B39" s="45"/>
       <c r="C39" s="11" t="s">
         <v>64</v>
       </c>
@@ -2331,10 +2418,13 @@
         <v>3</v>
       </c>
       <c r="F39" s="11"/>
-    </row>
-    <row r="40" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A40" s="37"/>
-      <c r="B40" s="39"/>
+      <c r="G39" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A40" s="52"/>
+      <c r="B40" s="46"/>
       <c r="C40" s="11" t="s">
         <v>65</v>
       </c>
@@ -2345,12 +2435,15 @@
         <v>3</v>
       </c>
       <c r="F40" s="11"/>
-    </row>
-    <row r="41" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A41" s="36" t="s">
+      <c r="G40" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A41" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="B41" s="38" t="s">
+      <c r="B41" s="53" t="s">
         <v>68</v>
       </c>
       <c r="C41" s="11" t="s">
@@ -2363,10 +2456,13 @@
         <v>15</v>
       </c>
       <c r="F41" s="11"/>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A42" s="40"/>
-      <c r="B42" s="41"/>
+      <c r="G41" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A42" s="51"/>
+      <c r="B42" s="45"/>
       <c r="C42" s="11" t="s">
         <v>70</v>
       </c>
@@ -2377,10 +2473,13 @@
         <v>10</v>
       </c>
       <c r="F42" s="11"/>
-    </row>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A43" s="37"/>
-      <c r="B43" s="39"/>
+      <c r="G42" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A43" s="52"/>
+      <c r="B43" s="46"/>
       <c r="C43" s="11" t="s">
         <v>71</v>
       </c>
@@ -2391,8 +2490,11 @@
         <v>3</v>
       </c>
       <c r="F43" s="11"/>
-    </row>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G43" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1">
       <c r="A44" s="5" t="s">
         <v>72</v>
       </c>
@@ -2409,12 +2511,15 @@
         <v>15</v>
       </c>
       <c r="F44" s="20"/>
-    </row>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A45" s="36" t="s">
+      <c r="G44" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A45" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="B45" s="38" t="s">
+      <c r="B45" s="53" t="s">
         <v>76</v>
       </c>
       <c r="C45" s="11" t="s">
@@ -2427,10 +2532,13 @@
         <v>3</v>
       </c>
       <c r="F45" s="11"/>
-    </row>
-    <row r="46" spans="1:6" ht="36" customHeight="1">
-      <c r="A46" s="37"/>
-      <c r="B46" s="39"/>
+      <c r="G45" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="36" customHeight="1">
+      <c r="A46" s="52"/>
+      <c r="B46" s="46"/>
       <c r="C46" s="11" t="s">
         <v>78</v>
       </c>
@@ -2441,12 +2549,15 @@
         <v>3</v>
       </c>
       <c r="F46" s="11"/>
-    </row>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A47" s="36" t="s">
+      <c r="G46" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A47" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="B47" s="38" t="s">
+      <c r="B47" s="53" t="s">
         <v>80</v>
       </c>
       <c r="C47" s="11" t="s">
@@ -2459,10 +2570,13 @@
         <v>15</v>
       </c>
       <c r="F47" s="11"/>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A48" s="40"/>
-      <c r="B48" s="41"/>
+      <c r="G47" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A48" s="51"/>
+      <c r="B48" s="45"/>
       <c r="C48" s="11" t="s">
         <v>82</v>
       </c>
@@ -2473,10 +2587,13 @@
         <v>10</v>
       </c>
       <c r="F48" s="11"/>
-    </row>
-    <row r="49" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A49" s="37"/>
-      <c r="B49" s="39"/>
+      <c r="G48" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A49" s="52"/>
+      <c r="B49" s="46"/>
       <c r="C49" s="11" t="s">
         <v>83</v>
       </c>
@@ -2487,8 +2604,11 @@
         <v>10</v>
       </c>
       <c r="F49" s="11"/>
-    </row>
-    <row r="50" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G49" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="38.25">
       <c r="A50" s="5" t="s">
         <v>84</v>
       </c>
@@ -2505,12 +2625,15 @@
         <v>5</v>
       </c>
       <c r="F50" s="11"/>
-    </row>
-    <row r="51" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A51" s="36" t="s">
+      <c r="G50" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A51" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="B51" s="38" t="s">
+      <c r="B51" s="53" t="s">
         <v>88</v>
       </c>
       <c r="C51" s="11" t="s">
@@ -2523,10 +2646,13 @@
         <v>2</v>
       </c>
       <c r="F51" s="11"/>
-    </row>
-    <row r="52" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A52" s="40"/>
-      <c r="B52" s="41"/>
+      <c r="G51" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A52" s="51"/>
+      <c r="B52" s="45"/>
       <c r="C52" s="11" t="s">
         <v>90</v>
       </c>
@@ -2537,10 +2663,13 @@
         <v>3</v>
       </c>
       <c r="F52" s="11"/>
-    </row>
-    <row r="53" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A53" s="40"/>
-      <c r="B53" s="41"/>
+      <c r="G52" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A53" s="51"/>
+      <c r="B53" s="45"/>
       <c r="C53" s="11" t="s">
         <v>91</v>
       </c>
@@ -2551,10 +2680,13 @@
         <v>5</v>
       </c>
       <c r="F53" s="11"/>
-    </row>
-    <row r="54" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A54" s="37"/>
-      <c r="B54" s="39"/>
+      <c r="G53" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A54" s="52"/>
+      <c r="B54" s="46"/>
       <c r="C54" s="11" t="s">
         <v>92</v>
       </c>
@@ -2565,8 +2697,11 @@
         <v>20</v>
       </c>
       <c r="F54" s="11"/>
-    </row>
-    <row r="55" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G54" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="38.25">
       <c r="A55" s="5" t="s">
         <v>93</v>
       </c>
@@ -2583,8 +2718,11 @@
         <v>5</v>
       </c>
       <c r="F55" s="11"/>
-    </row>
-    <row r="56" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G55" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="25.5">
       <c r="A56" s="5" t="s">
         <v>96</v>
       </c>
@@ -2601,8 +2739,11 @@
         <v>3</v>
       </c>
       <c r="F56" s="11"/>
-    </row>
-    <row r="57" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G56" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="25.5">
       <c r="A57" s="5" t="s">
         <v>99</v>
       </c>
@@ -2619,8 +2760,11 @@
         <v>2</v>
       </c>
       <c r="F57" s="11"/>
-    </row>
-    <row r="58" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G57" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="25.5">
       <c r="A58" s="8" t="s">
         <v>102</v>
       </c>
@@ -2637,18 +2781,21 @@
         <v>2</v>
       </c>
       <c r="F58" s="14"/>
-    </row>
-    <row r="59" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A59" s="42" t="s">
+      <c r="G58" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A59" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="B59" s="43"/>
-      <c r="C59" s="43"/>
-      <c r="D59" s="43"/>
-      <c r="E59" s="43"/>
-      <c r="F59" s="44"/>
-    </row>
-    <row r="60" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B59" s="55"/>
+      <c r="C59" s="55"/>
+      <c r="D59" s="55"/>
+      <c r="E59" s="55"/>
+      <c r="F59" s="56"/>
+    </row>
+    <row r="60" spans="1:7" ht="15.75" customHeight="1">
       <c r="A60" s="5" t="s">
         <v>9</v>
       </c>
@@ -2665,8 +2812,11 @@
         <v>15</v>
       </c>
       <c r="F60" s="11"/>
-    </row>
-    <row r="61" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G60" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="25.5">
       <c r="A61" s="5" t="s">
         <v>12</v>
       </c>
@@ -2683,12 +2833,15 @@
         <v>15</v>
       </c>
       <c r="F61" s="11"/>
-    </row>
-    <row r="62" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A62" s="36" t="s">
+      <c r="G61" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A62" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B62" s="38" t="s">
+      <c r="B62" s="53" t="s">
         <v>110</v>
       </c>
       <c r="C62" s="11" t="s">
@@ -2701,10 +2854,13 @@
         <v>5</v>
       </c>
       <c r="F62" s="11"/>
-    </row>
-    <row r="63" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A63" s="37"/>
-      <c r="B63" s="39"/>
+      <c r="G62" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A63" s="52"/>
+      <c r="B63" s="46"/>
       <c r="C63" s="11" t="s">
         <v>112</v>
       </c>
@@ -2715,8 +2871,11 @@
         <v>2</v>
       </c>
       <c r="F63" s="11"/>
-    </row>
-    <row r="64" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G63" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="25.5">
       <c r="A64" s="5" t="s">
         <v>32</v>
       </c>
@@ -2733,12 +2892,15 @@
         <v>5</v>
       </c>
       <c r="F64" s="11"/>
-    </row>
-    <row r="65" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A65" s="36" t="s">
+      <c r="G64" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A65" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B65" s="38" t="s">
+      <c r="B65" s="53" t="s">
         <v>115</v>
       </c>
       <c r="C65" s="11" t="s">
@@ -2751,10 +2913,13 @@
         <v>5</v>
       </c>
       <c r="F65" s="11"/>
-    </row>
-    <row r="66" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A66" s="40"/>
-      <c r="B66" s="41"/>
+      <c r="G65" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A66" s="51"/>
+      <c r="B66" s="45"/>
       <c r="C66" s="11" t="s">
         <v>117</v>
       </c>
@@ -2765,10 +2930,13 @@
         <v>2</v>
       </c>
       <c r="F66" s="11"/>
-    </row>
-    <row r="67" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A67" s="37"/>
-      <c r="B67" s="39"/>
+      <c r="G66" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A67" s="52"/>
+      <c r="B67" s="46"/>
       <c r="C67" s="11" t="s">
         <v>118</v>
       </c>
@@ -2779,8 +2947,11 @@
         <v>2</v>
       </c>
       <c r="F67" s="11"/>
-    </row>
-    <row r="68" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G67" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="25.5">
       <c r="A68" s="5" t="s">
         <v>17</v>
       </c>
@@ -2797,8 +2968,11 @@
         <v>3</v>
       </c>
       <c r="F68" s="11"/>
-    </row>
-    <row r="69" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G68" s="37" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="25.5">
       <c r="A69" s="5" t="s">
         <v>72</v>
       </c>
@@ -2815,8 +2989,11 @@
         <v>5</v>
       </c>
       <c r="F69" s="11"/>
-    </row>
-    <row r="70" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G69" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="38.25">
       <c r="A70" s="8" t="s">
         <v>93</v>
       </c>
@@ -2833,18 +3010,21 @@
         <v>5</v>
       </c>
       <c r="F70" s="14"/>
-    </row>
-    <row r="71" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A71" s="42" t="s">
+      <c r="G70" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A71" s="54" t="s">
         <v>125</v>
       </c>
-      <c r="B71" s="43"/>
-      <c r="C71" s="43"/>
-      <c r="D71" s="43"/>
-      <c r="E71" s="43"/>
-      <c r="F71" s="44"/>
-    </row>
-    <row r="72" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B71" s="55"/>
+      <c r="C71" s="55"/>
+      <c r="D71" s="55"/>
+      <c r="E71" s="55"/>
+      <c r="F71" s="56"/>
+    </row>
+    <row r="72" spans="1:7" ht="25.5">
       <c r="A72" s="5" t="s">
         <v>9</v>
       </c>
@@ -2861,8 +3041,11 @@
         <v>5</v>
       </c>
       <c r="F72" s="11"/>
-    </row>
-    <row r="73" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G72" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="25.5">
       <c r="A73" s="5" t="s">
         <v>12</v>
       </c>
@@ -2879,8 +3062,11 @@
         <v>5</v>
       </c>
       <c r="F73" s="11"/>
-    </row>
-    <row r="74" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G73" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="25.5">
       <c r="A74" s="5" t="s">
         <v>17</v>
       </c>
@@ -2897,8 +3083,11 @@
         <v>5</v>
       </c>
       <c r="F74" s="11"/>
-    </row>
-    <row r="75" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G74" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="25.5">
       <c r="A75" s="5" t="s">
         <v>72</v>
       </c>
@@ -2915,8 +3104,11 @@
         <v>2</v>
       </c>
       <c r="F75" s="11"/>
-    </row>
-    <row r="76" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G75" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="12.75">
       <c r="A76" s="5" t="s">
         <v>75</v>
       </c>
@@ -2933,8 +3125,11 @@
         <v>3</v>
       </c>
       <c r="F76" s="11"/>
-    </row>
-    <row r="77" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G76" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="12.75">
       <c r="A77" s="5" t="s">
         <v>79</v>
       </c>
@@ -2951,8 +3146,11 @@
         <v>3</v>
       </c>
       <c r="F77" s="11"/>
-    </row>
-    <row r="78" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G77" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="51">
       <c r="A78" s="8" t="s">
         <v>84</v>
       </c>
@@ -2969,18 +3167,21 @@
         <v>15</v>
       </c>
       <c r="F78" s="14"/>
-    </row>
-    <row r="79" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A79" s="42" t="s">
+      <c r="G78" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="16.5">
+      <c r="A79" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="B79" s="43"/>
-      <c r="C79" s="43"/>
-      <c r="D79" s="43"/>
-      <c r="E79" s="43"/>
-      <c r="F79" s="44"/>
-    </row>
-    <row r="80" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B79" s="55"/>
+      <c r="C79" s="55"/>
+      <c r="D79" s="55"/>
+      <c r="E79" s="55"/>
+      <c r="F79" s="56"/>
+    </row>
+    <row r="80" spans="1:7" ht="25.5">
       <c r="A80" s="5" t="s">
         <v>9</v>
       </c>
@@ -2997,8 +3198,11 @@
         <v>10</v>
       </c>
       <c r="F80" s="23"/>
-    </row>
-    <row r="81" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G80" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="25.5">
       <c r="A81" s="5" t="s">
         <v>12</v>
       </c>
@@ -3015,134 +3219,164 @@
         <v>5</v>
       </c>
       <c r="F81" s="23"/>
-    </row>
-    <row r="82" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G81" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="12.75">
       <c r="A82" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="C82" s="61" t="s">
+      <c r="C82" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="D82" s="54"/>
-      <c r="E82" s="54"/>
+      <c r="D82" s="62"/>
+      <c r="E82" s="62"/>
       <c r="F82" s="24"/>
-    </row>
-    <row r="83" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G82" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="12.75">
       <c r="A83" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C83" s="46"/>
-      <c r="D83" s="46"/>
-      <c r="E83" s="46"/>
+      <c r="C83" s="39"/>
+      <c r="D83" s="39"/>
+      <c r="E83" s="39"/>
       <c r="F83" s="25"/>
-    </row>
-    <row r="84" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G83" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="25.5">
       <c r="A84" s="5" t="s">
         <v>145</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="C84" s="46"/>
-      <c r="D84" s="46"/>
-      <c r="E84" s="46"/>
+      <c r="C84" s="39"/>
+      <c r="D84" s="39"/>
+      <c r="E84" s="39"/>
       <c r="F84" s="25"/>
-    </row>
-    <row r="85" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G84" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" ht="25.5">
       <c r="A85" s="5" t="s">
         <v>147</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="C85" s="46"/>
-      <c r="D85" s="46"/>
-      <c r="E85" s="46"/>
+      <c r="C85" s="39"/>
+      <c r="D85" s="39"/>
+      <c r="E85" s="39"/>
       <c r="F85" s="25"/>
-    </row>
-    <row r="86" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G85" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="12.75">
       <c r="A86" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="C86" s="46"/>
-      <c r="D86" s="46"/>
-      <c r="E86" s="46"/>
+      <c r="C86" s="39"/>
+      <c r="D86" s="39"/>
+      <c r="E86" s="39"/>
       <c r="F86" s="25"/>
-    </row>
-    <row r="87" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G86" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" ht="25.5">
       <c r="A87" s="5" t="s">
         <v>150</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="C87" s="46"/>
-      <c r="D87" s="46"/>
-      <c r="E87" s="46"/>
+      <c r="C87" s="39"/>
+      <c r="D87" s="39"/>
+      <c r="E87" s="39"/>
       <c r="F87" s="25"/>
-    </row>
-    <row r="88" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G87" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" ht="12.75">
       <c r="A88" s="8" t="s">
         <v>152</v>
       </c>
       <c r="B88" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C88" s="47"/>
-      <c r="D88" s="47"/>
-      <c r="E88" s="47"/>
+      <c r="C88" s="40"/>
+      <c r="D88" s="40"/>
+      <c r="E88" s="40"/>
       <c r="F88" s="25"/>
-    </row>
-    <row r="89" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A89" s="42" t="s">
+      <c r="G88" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="16.5">
+      <c r="A89" s="54" t="s">
         <v>154</v>
       </c>
-      <c r="B89" s="43"/>
-      <c r="C89" s="43"/>
-      <c r="D89" s="43"/>
-      <c r="E89" s="43"/>
-      <c r="F89" s="44"/>
-    </row>
-    <row r="90" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B89" s="55"/>
+      <c r="C89" s="55"/>
+      <c r="D89" s="55"/>
+      <c r="E89" s="55"/>
+      <c r="F89" s="56"/>
+    </row>
+    <row r="90" spans="1:7" ht="38.25">
       <c r="A90" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="C90" s="45" t="s">
+      <c r="C90" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="D90" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E90" s="51">
+      <c r="D90" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E90" s="44">
         <v>15</v>
       </c>
-      <c r="F90" s="45"/>
-    </row>
-    <row r="91" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F90" s="38"/>
+      <c r="G90" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="38.25">
       <c r="A91" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B91" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C91" s="47"/>
-      <c r="D91" s="50"/>
-      <c r="E91" s="39"/>
-      <c r="F91" s="47"/>
-    </row>
-    <row r="92" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C91" s="40"/>
+      <c r="D91" s="43"/>
+      <c r="E91" s="46"/>
+      <c r="F91" s="40"/>
+      <c r="G91" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="89.25">
       <c r="A92" s="5" t="s">
         <v>17</v>
       </c>
@@ -3159,8 +3393,11 @@
         <v>30</v>
       </c>
       <c r="F92" s="11"/>
-    </row>
-    <row r="93" spans="1:6" ht="28.5" customHeight="1">
+      <c r="G92" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="25.5">
       <c r="A93" s="8" t="s">
         <v>72</v>
       </c>
@@ -3177,22 +3414,25 @@
         <v>5</v>
       </c>
       <c r="F93" s="14"/>
-    </row>
-    <row r="94" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A94" s="42" t="s">
+      <c r="G93" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="16.5">
+      <c r="A94" s="54" t="s">
         <v>162</v>
       </c>
-      <c r="B94" s="43"/>
-      <c r="C94" s="43"/>
-      <c r="D94" s="43"/>
-      <c r="E94" s="43"/>
-      <c r="F94" s="44"/>
-    </row>
-    <row r="95" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A95" s="36" t="s">
+      <c r="B94" s="55"/>
+      <c r="C94" s="55"/>
+      <c r="D94" s="55"/>
+      <c r="E94" s="55"/>
+      <c r="F94" s="56"/>
+    </row>
+    <row r="95" spans="1:7" ht="12.75">
+      <c r="A95" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B95" s="38" t="s">
+      <c r="B95" s="53" t="s">
         <v>163</v>
       </c>
       <c r="C95" s="11" t="s">
@@ -3205,10 +3445,13 @@
         <v>15</v>
       </c>
       <c r="F95" s="11"/>
-    </row>
-    <row r="96" spans="1:6" ht="72.75" customHeight="1">
-      <c r="A96" s="37"/>
-      <c r="B96" s="39"/>
+      <c r="G95" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="12.75">
+      <c r="A96" s="52"/>
+      <c r="B96" s="46"/>
       <c r="C96" s="11" t="s">
         <v>165</v>
       </c>
@@ -3219,74 +3462,92 @@
         <v>3</v>
       </c>
       <c r="F96" s="11"/>
-    </row>
-    <row r="97" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G96" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="51">
       <c r="A97" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B97" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="C97" s="45" t="s">
+      <c r="C97" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="D97" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E97" s="51">
+      <c r="D97" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E97" s="44">
         <v>20</v>
       </c>
-      <c r="F97" s="45"/>
-    </row>
-    <row r="98" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F97" s="38"/>
+      <c r="G97" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="51">
       <c r="A98" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B98" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="C98" s="46"/>
-      <c r="D98" s="49"/>
-      <c r="E98" s="41"/>
-      <c r="F98" s="46"/>
-    </row>
-    <row r="99" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C98" s="39"/>
+      <c r="D98" s="42"/>
+      <c r="E98" s="45"/>
+      <c r="F98" s="39"/>
+      <c r="G98" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="38.25">
       <c r="A99" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B99" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="C99" s="46"/>
-      <c r="D99" s="49"/>
-      <c r="E99" s="41"/>
-      <c r="F99" s="46"/>
-    </row>
-    <row r="100" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C99" s="39"/>
+      <c r="D99" s="42"/>
+      <c r="E99" s="45"/>
+      <c r="F99" s="39"/>
+      <c r="G99" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" ht="63.75">
       <c r="A100" s="5" t="s">
         <v>93</v>
       </c>
       <c r="B100" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="C100" s="46"/>
-      <c r="D100" s="49"/>
-      <c r="E100" s="41"/>
-      <c r="F100" s="46"/>
-    </row>
-    <row r="101" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C100" s="39"/>
+      <c r="D100" s="42"/>
+      <c r="E100" s="45"/>
+      <c r="F100" s="39"/>
+      <c r="G100" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="63.75">
       <c r="A101" s="5" t="s">
         <v>171</v>
       </c>
       <c r="B101" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="C101" s="47"/>
-      <c r="D101" s="50"/>
-      <c r="E101" s="39"/>
-      <c r="F101" s="47"/>
-    </row>
-    <row r="102" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C101" s="40"/>
+      <c r="D101" s="43"/>
+      <c r="E101" s="46"/>
+      <c r="F101" s="40"/>
+      <c r="G101" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="38.25">
       <c r="A102" s="5" t="s">
         <v>173</v>
       </c>
@@ -3303,8 +3564,11 @@
         <v>5</v>
       </c>
       <c r="F102" s="11"/>
-    </row>
-    <row r="103" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G102" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="76.5">
       <c r="A103" s="5" t="s">
         <v>175</v>
       </c>
@@ -3321,8 +3585,11 @@
         <v>5</v>
       </c>
       <c r="F103" s="11"/>
-    </row>
-    <row r="104" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G103" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="63.75">
       <c r="A104" s="5" t="s">
         <v>177</v>
       </c>
@@ -3339,8 +3606,11 @@
         <v>4</v>
       </c>
       <c r="F104" s="11"/>
-    </row>
-    <row r="105" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G104" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" ht="51">
       <c r="A105" s="5" t="s">
         <v>180</v>
       </c>
@@ -3357,8 +3627,11 @@
         <v>1</v>
       </c>
       <c r="F105" s="11"/>
-    </row>
-    <row r="106" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G105" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="12.75">
       <c r="A106" s="5" t="s">
         <v>182</v>
       </c>
@@ -3375,8 +3648,11 @@
         <v>10</v>
       </c>
       <c r="F106" s="11"/>
-    </row>
-    <row r="107" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G106" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="38.25">
       <c r="A107" s="5" t="s">
         <v>184</v>
       </c>
@@ -3393,8 +3669,11 @@
         <v>2</v>
       </c>
       <c r="F107" s="11"/>
-    </row>
-    <row r="108" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G107" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="25.5">
       <c r="A108" s="5" t="s">
         <v>187</v>
       </c>
@@ -3411,8 +3690,11 @@
         <v>2</v>
       </c>
       <c r="F108" s="11"/>
-    </row>
-    <row r="109" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G108" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="51">
       <c r="A109" s="5" t="s">
         <v>189</v>
       </c>
@@ -3429,12 +3711,15 @@
         <v>3</v>
       </c>
       <c r="F109" s="11"/>
-    </row>
-    <row r="110" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A110" s="36" t="s">
+      <c r="G109" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="12.75">
+      <c r="A110" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="B110" s="38" t="s">
+      <c r="B110" s="53" t="s">
         <v>192</v>
       </c>
       <c r="C110" s="11" t="s">
@@ -3447,10 +3732,13 @@
         <v>5</v>
       </c>
       <c r="F110" s="11"/>
-    </row>
-    <row r="111" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A111" s="40"/>
-      <c r="B111" s="41"/>
+      <c r="G110" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="12.75">
+      <c r="A111" s="51"/>
+      <c r="B111" s="45"/>
       <c r="C111" s="11" t="s">
         <v>193</v>
       </c>
@@ -3461,10 +3749,13 @@
         <v>10</v>
       </c>
       <c r="F111" s="11"/>
-    </row>
-    <row r="112" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A112" s="37"/>
-      <c r="B112" s="39"/>
+      <c r="G111" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" ht="12.75">
+      <c r="A112" s="52"/>
+      <c r="B112" s="46"/>
       <c r="C112" s="11" t="s">
         <v>194</v>
       </c>
@@ -3475,12 +3766,15 @@
         <v>10</v>
       </c>
       <c r="F112" s="11"/>
-    </row>
-    <row r="113" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A113" s="36" t="s">
+      <c r="G112" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="12.75">
+      <c r="A113" s="50" t="s">
         <v>195</v>
       </c>
-      <c r="B113" s="38" t="s">
+      <c r="B113" s="53" t="s">
         <v>196</v>
       </c>
       <c r="C113" s="11" t="s">
@@ -3493,10 +3787,13 @@
         <v>5</v>
       </c>
       <c r="F113" s="11"/>
-    </row>
-    <row r="114" spans="1:6" ht="41.25" customHeight="1">
-      <c r="A114" s="37"/>
-      <c r="B114" s="39"/>
+      <c r="G113" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="12.75">
+      <c r="A114" s="52"/>
+      <c r="B114" s="46"/>
       <c r="C114" s="11" t="s">
         <v>197</v>
       </c>
@@ -3507,8 +3804,11 @@
         <v>10</v>
       </c>
       <c r="F114" s="11"/>
-    </row>
-    <row r="115" spans="1:6" ht="84" customHeight="1">
+      <c r="G114" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="76.5">
       <c r="A115" s="8" t="s">
         <v>198</v>
       </c>
@@ -3525,94 +3825,112 @@
         <v>4</v>
       </c>
       <c r="F115" s="14"/>
-    </row>
-    <row r="116" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A116" s="42" t="s">
+      <c r="G115" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="16.5">
+      <c r="A116" s="54" t="s">
         <v>200</v>
       </c>
-      <c r="B116" s="43"/>
-      <c r="C116" s="43"/>
-      <c r="D116" s="43"/>
-      <c r="E116" s="43"/>
-      <c r="F116" s="44"/>
-    </row>
-    <row r="117" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B116" s="55"/>
+      <c r="C116" s="55"/>
+      <c r="D116" s="55"/>
+      <c r="E116" s="55"/>
+      <c r="F116" s="56"/>
+    </row>
+    <row r="117" spans="1:7" ht="38.25">
       <c r="A117" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B117" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="C117" s="45" t="s">
+      <c r="C117" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="D117" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E117" s="51">
+      <c r="D117" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E117" s="44">
         <v>5</v>
       </c>
-      <c r="F117" s="45"/>
-    </row>
-    <row r="118" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F117" s="38"/>
+      <c r="G117" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" ht="51">
       <c r="A118" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B118" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C118" s="47"/>
-      <c r="D118" s="52"/>
-      <c r="E118" s="39"/>
-      <c r="F118" s="47"/>
-    </row>
-    <row r="119" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C118" s="40"/>
+      <c r="D118" s="48"/>
+      <c r="E118" s="46"/>
+      <c r="F118" s="40"/>
+      <c r="G118" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="25.5">
       <c r="A119" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B119" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="C119" s="45" t="s">
+      <c r="C119" s="38" t="s">
         <v>202</v>
       </c>
       <c r="D119" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E119" s="51">
+      <c r="E119" s="44">
         <v>15</v>
       </c>
-      <c r="F119" s="45"/>
-    </row>
-    <row r="120" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F119" s="38"/>
+      <c r="G119" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="12.75">
       <c r="A120" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B120" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C120" s="46"/>
+      <c r="C120" s="39"/>
       <c r="D120" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E120" s="41"/>
-      <c r="F120" s="46"/>
-    </row>
-    <row r="121" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E120" s="45"/>
+      <c r="F120" s="39"/>
+      <c r="G120" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="51">
       <c r="A121" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B121" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="C121" s="47"/>
+      <c r="C121" s="40"/>
       <c r="D121" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E121" s="39"/>
-      <c r="F121" s="47"/>
-    </row>
-    <row r="122" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E121" s="46"/>
+      <c r="F121" s="40"/>
+      <c r="G121" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="38.25">
       <c r="A122" s="8" t="s">
         <v>72</v>
       </c>
@@ -3629,60 +3947,72 @@
         <v>5</v>
       </c>
       <c r="F122" s="14"/>
-    </row>
-    <row r="123" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A123" s="42" t="s">
+      <c r="G122" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" ht="16.5">
+      <c r="A123" s="54" t="s">
         <v>208</v>
       </c>
-      <c r="B123" s="43"/>
-      <c r="C123" s="43"/>
-      <c r="D123" s="43"/>
-      <c r="E123" s="43"/>
-      <c r="F123" s="44"/>
-    </row>
-    <row r="124" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B123" s="55"/>
+      <c r="C123" s="55"/>
+      <c r="D123" s="55"/>
+      <c r="E123" s="55"/>
+      <c r="F123" s="56"/>
+    </row>
+    <row r="124" spans="1:7" ht="38.25">
       <c r="A124" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B124" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="C124" s="45" t="s">
+      <c r="C124" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="D124" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E124" s="51">
+      <c r="D124" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E124" s="44">
         <v>15</v>
       </c>
-      <c r="F124" s="45"/>
-    </row>
-    <row r="125" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F124" s="38"/>
+      <c r="G124" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="12.75">
       <c r="A125" s="5" t="s">
         <v>210</v>
       </c>
       <c r="B125" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="C125" s="46"/>
-      <c r="D125" s="49"/>
-      <c r="E125" s="41"/>
-      <c r="F125" s="46"/>
-    </row>
-    <row r="126" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C125" s="39"/>
+      <c r="D125" s="42"/>
+      <c r="E125" s="45"/>
+      <c r="F125" s="39"/>
+      <c r="G125" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" ht="25.5">
       <c r="A126" s="5" t="s">
         <v>212</v>
       </c>
       <c r="B126" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="C126" s="47"/>
-      <c r="D126" s="50"/>
-      <c r="E126" s="39"/>
-      <c r="F126" s="47"/>
-    </row>
-    <row r="127" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C126" s="40"/>
+      <c r="D126" s="43"/>
+      <c r="E126" s="46"/>
+      <c r="F126" s="40"/>
+      <c r="G126" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" ht="51">
       <c r="A127" s="5" t="s">
         <v>214</v>
       </c>
@@ -3699,8 +4029,11 @@
         <v>5</v>
       </c>
       <c r="F127" s="11"/>
-    </row>
-    <row r="128" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G127" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" ht="51">
       <c r="A128" s="5" t="s">
         <v>216</v>
       </c>
@@ -3717,94 +4050,115 @@
         <v>5</v>
       </c>
       <c r="F128" s="11"/>
-    </row>
-    <row r="129" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G128" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" ht="51">
       <c r="A129" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B129" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="C129" s="45" t="s">
+      <c r="C129" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="D129" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E129" s="51">
+      <c r="D129" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E129" s="44">
         <v>10</v>
       </c>
-      <c r="F129" s="45"/>
-    </row>
-    <row r="130" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F129" s="38"/>
+      <c r="G129" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" ht="25.5">
       <c r="A130" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B130" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="C130" s="46"/>
-      <c r="D130" s="49"/>
-      <c r="E130" s="41"/>
-      <c r="F130" s="46"/>
-    </row>
-    <row r="131" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C130" s="39"/>
+      <c r="D130" s="42"/>
+      <c r="E130" s="45"/>
+      <c r="F130" s="39"/>
+      <c r="G130" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" ht="12.75">
       <c r="A131" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B131" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="C131" s="47"/>
-      <c r="D131" s="50"/>
-      <c r="E131" s="39"/>
-      <c r="F131" s="47"/>
-    </row>
-    <row r="132" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C131" s="40"/>
+      <c r="D131" s="43"/>
+      <c r="E131" s="46"/>
+      <c r="F131" s="40"/>
+      <c r="G131" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="25.5">
       <c r="A132" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B132" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="C132" s="45" t="s">
+      <c r="C132" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="D132" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E132" s="51">
+      <c r="D132" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E132" s="44">
         <v>10</v>
       </c>
-      <c r="F132" s="45"/>
-    </row>
-    <row r="133" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F132" s="38"/>
+      <c r="G132" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="25.5">
       <c r="A133" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B133" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="C133" s="46"/>
-      <c r="D133" s="49"/>
-      <c r="E133" s="41"/>
-      <c r="F133" s="46"/>
-    </row>
-    <row r="134" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A134" s="36" t="s">
+      <c r="C133" s="39"/>
+      <c r="D133" s="42"/>
+      <c r="E133" s="45"/>
+      <c r="F133" s="39"/>
+      <c r="G133" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" ht="12.75">
+      <c r="A134" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="B134" s="38" t="s">
+      <c r="B134" s="53" t="s">
         <v>222</v>
       </c>
-      <c r="C134" s="47"/>
-      <c r="D134" s="50"/>
-      <c r="E134" s="39"/>
-      <c r="F134" s="47"/>
-    </row>
-    <row r="135" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A135" s="40"/>
-      <c r="B135" s="41"/>
+      <c r="C134" s="40"/>
+      <c r="D134" s="43"/>
+      <c r="E134" s="46"/>
+      <c r="F134" s="40"/>
+      <c r="G134" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="12.75">
+      <c r="A135" s="51"/>
+      <c r="B135" s="45"/>
       <c r="C135" s="11" t="s">
         <v>223</v>
       </c>
@@ -3815,10 +4169,13 @@
         <v>10</v>
       </c>
       <c r="F135" s="11"/>
-    </row>
-    <row r="136" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A136" s="40"/>
-      <c r="B136" s="41"/>
+      <c r="G135" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" ht="12.75">
+      <c r="A136" s="51"/>
+      <c r="B136" s="45"/>
       <c r="C136" s="11" t="s">
         <v>224</v>
       </c>
@@ -3829,10 +4186,13 @@
         <v>20</v>
       </c>
       <c r="F136" s="11"/>
-    </row>
-    <row r="137" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A137" s="37"/>
-      <c r="B137" s="39"/>
+      <c r="G136" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="12.75">
+      <c r="A137" s="52"/>
+      <c r="B137" s="46"/>
       <c r="C137" s="11" t="s">
         <v>225</v>
       </c>
@@ -3843,12 +4203,15 @@
         <v>25</v>
       </c>
       <c r="F137" s="11"/>
-    </row>
-    <row r="138" spans="1:6" ht="24" customHeight="1">
-      <c r="A138" s="36" t="s">
+      <c r="G137" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="12.75">
+      <c r="A138" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="B138" s="38" t="s">
+      <c r="B138" s="53" t="s">
         <v>226</v>
       </c>
       <c r="C138" s="11" t="s">
@@ -3861,10 +4224,13 @@
         <v>15</v>
       </c>
       <c r="F138" s="11"/>
-    </row>
-    <row r="139" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A139" s="40"/>
-      <c r="B139" s="41"/>
+      <c r="G138" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" ht="12.75">
+      <c r="A139" s="51"/>
+      <c r="B139" s="45"/>
       <c r="C139" s="11" t="s">
         <v>227</v>
       </c>
@@ -3875,10 +4241,13 @@
         <v>15</v>
       </c>
       <c r="F139" s="11"/>
-    </row>
-    <row r="140" spans="1:6" ht="32.25" customHeight="1">
-      <c r="A140" s="37"/>
-      <c r="B140" s="39"/>
+      <c r="G139" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="12.75">
+      <c r="A140" s="52"/>
+      <c r="B140" s="46"/>
       <c r="C140" s="14" t="s">
         <v>228</v>
       </c>
@@ -3889,126 +4258,153 @@
         <v>20</v>
       </c>
       <c r="F140" s="14"/>
-    </row>
-    <row r="141" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A141" s="42" t="s">
+      <c r="G140" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="16.5">
+      <c r="A141" s="54" t="s">
         <v>229</v>
       </c>
-      <c r="B141" s="43"/>
-      <c r="C141" s="43"/>
-      <c r="D141" s="43"/>
-      <c r="E141" s="43"/>
-      <c r="F141" s="44"/>
-    </row>
-    <row r="142" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B141" s="55"/>
+      <c r="C141" s="55"/>
+      <c r="D141" s="55"/>
+      <c r="E141" s="55"/>
+      <c r="F141" s="56"/>
+    </row>
+    <row r="142" spans="1:7" ht="25.5">
       <c r="A142" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B142" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="C142" s="45" t="s">
+      <c r="C142" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="D142" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E142" s="51">
+      <c r="D142" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E142" s="44">
         <v>100</v>
       </c>
-      <c r="F142" s="45"/>
-    </row>
-    <row r="143" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F142" s="38"/>
+      <c r="G142" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="25.5">
       <c r="A143" s="5" t="s">
         <v>210</v>
       </c>
       <c r="B143" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="C143" s="46"/>
-      <c r="D143" s="49"/>
-      <c r="E143" s="41"/>
-      <c r="F143" s="46"/>
-    </row>
-    <row r="144" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C143" s="39"/>
+      <c r="D143" s="42"/>
+      <c r="E143" s="45"/>
+      <c r="F143" s="39"/>
+      <c r="G143" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="25.5">
       <c r="A144" s="5" t="s">
         <v>212</v>
       </c>
       <c r="B144" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="C144" s="46"/>
-      <c r="D144" s="49"/>
-      <c r="E144" s="41"/>
-      <c r="F144" s="46"/>
-    </row>
-    <row r="145" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C144" s="39"/>
+      <c r="D144" s="42"/>
+      <c r="E144" s="45"/>
+      <c r="F144" s="39"/>
+      <c r="G144" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="63.75">
       <c r="A145" s="5" t="s">
         <v>214</v>
       </c>
       <c r="B145" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="C145" s="47"/>
-      <c r="D145" s="50"/>
-      <c r="E145" s="39"/>
-      <c r="F145" s="47"/>
-    </row>
-    <row r="146" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C145" s="40"/>
+      <c r="D145" s="43"/>
+      <c r="E145" s="46"/>
+      <c r="F145" s="40"/>
+      <c r="G145" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="25.5">
       <c r="A146" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B146" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="C146" s="45" t="s">
+      <c r="C146" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="D146" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E146" s="51">
+      <c r="D146" s="41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E146" s="44">
         <v>100</v>
       </c>
-      <c r="F146" s="45"/>
-    </row>
-    <row r="147" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F146" s="38"/>
+      <c r="G146" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="25.5">
       <c r="A147" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B147" s="17" t="s">
         <v>235</v>
       </c>
-      <c r="C147" s="46"/>
-      <c r="D147" s="49"/>
-      <c r="E147" s="41"/>
-      <c r="F147" s="46"/>
-    </row>
-    <row r="148" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C147" s="39"/>
+      <c r="D147" s="42"/>
+      <c r="E147" s="45"/>
+      <c r="F147" s="39"/>
+      <c r="G147" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" ht="38.25">
       <c r="A148" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B148" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="C148" s="46"/>
-      <c r="D148" s="49"/>
-      <c r="E148" s="41"/>
-      <c r="F148" s="46"/>
-    </row>
-    <row r="149" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C148" s="39"/>
+      <c r="D148" s="42"/>
+      <c r="E148" s="45"/>
+      <c r="F148" s="39"/>
+      <c r="G148" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" ht="51">
       <c r="A149" s="26" t="s">
         <v>36</v>
       </c>
       <c r="B149" s="27" t="s">
         <v>237</v>
       </c>
-      <c r="C149" s="62"/>
-      <c r="D149" s="52"/>
-      <c r="E149" s="63"/>
-      <c r="F149" s="62"/>
-    </row>
-    <row r="150" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C149" s="47"/>
+      <c r="D149" s="48"/>
+      <c r="E149" s="49"/>
+      <c r="F149" s="47"/>
+      <c r="G149" s="37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" ht="15.75" customHeight="1">
       <c r="A150" s="28"/>
       <c r="B150" s="28"/>
       <c r="C150" s="29"/>
@@ -4021,7 +4417,7 @@
       </c>
       <c r="F150" s="29"/>
     </row>
-    <row r="151" spans="1:6" ht="15.75" customHeight="1">
+    <row r="151" spans="1:7" ht="15.75" customHeight="1">
       <c r="A151" s="28"/>
       <c r="B151" s="32"/>
       <c r="C151" s="29"/>
@@ -4036,15 +4432,15 @@
         <v>240</v>
       </c>
     </row>
-    <row r="152" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="153" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="154" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="155" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="156" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="157" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="158" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="159" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="160" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="152" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="153" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="154" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="155" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="156" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="157" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="158" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="159" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="160" spans="1:7" ht="15.75" customHeight="1"/>
     <row r="161" ht="15.75" customHeight="1"/>
     <row r="162" ht="15.75" customHeight="1"/>
     <row r="163" ht="15.75" customHeight="1"/>
@@ -4887,83 +5283,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="B51:B54"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A35:A40"/>
-    <mergeCell ref="B35:B40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="C4:E5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="C7:E9"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="A138:A140"/>
-    <mergeCell ref="B138:B140"/>
-    <mergeCell ref="A141:F141"/>
-    <mergeCell ref="C129:C131"/>
-    <mergeCell ref="D129:D131"/>
-    <mergeCell ref="E129:E131"/>
-    <mergeCell ref="F129:F131"/>
-    <mergeCell ref="C132:C134"/>
-    <mergeCell ref="F132:F134"/>
-    <mergeCell ref="D132:D134"/>
-    <mergeCell ref="E132:E134"/>
-    <mergeCell ref="C119:C121"/>
-    <mergeCell ref="E119:E121"/>
-    <mergeCell ref="F119:F121"/>
-    <mergeCell ref="A123:F123"/>
-    <mergeCell ref="C124:C126"/>
-    <mergeCell ref="F124:F126"/>
-    <mergeCell ref="D124:D126"/>
-    <mergeCell ref="E124:E126"/>
-    <mergeCell ref="A113:A114"/>
-    <mergeCell ref="B113:B114"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="C117:C118"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="F117:F118"/>
-    <mergeCell ref="C97:C101"/>
-    <mergeCell ref="D97:D101"/>
-    <mergeCell ref="E97:E101"/>
-    <mergeCell ref="F97:F101"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="B65:B67"/>
+    <mergeCell ref="A71:F71"/>
     <mergeCell ref="A79:F79"/>
     <mergeCell ref="A89:F89"/>
     <mergeCell ref="A94:F94"/>
@@ -4974,11 +5298,83 @@
     <mergeCell ref="D90:D91"/>
     <mergeCell ref="E90:E91"/>
     <mergeCell ref="F90:F91"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="B65:B67"/>
-    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="C97:C101"/>
+    <mergeCell ref="D97:D101"/>
+    <mergeCell ref="E97:E101"/>
+    <mergeCell ref="F97:F101"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="A113:A114"/>
+    <mergeCell ref="B113:B114"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="C117:C118"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="F117:F118"/>
+    <mergeCell ref="C119:C121"/>
+    <mergeCell ref="E119:E121"/>
+    <mergeCell ref="F119:F121"/>
+    <mergeCell ref="A123:F123"/>
+    <mergeCell ref="C124:C126"/>
+    <mergeCell ref="F124:F126"/>
+    <mergeCell ref="D124:D126"/>
+    <mergeCell ref="E124:E126"/>
+    <mergeCell ref="C129:C131"/>
+    <mergeCell ref="D129:D131"/>
+    <mergeCell ref="E129:E131"/>
+    <mergeCell ref="F129:F131"/>
+    <mergeCell ref="C132:C134"/>
+    <mergeCell ref="F132:F134"/>
+    <mergeCell ref="D132:D134"/>
+    <mergeCell ref="E132:E134"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="A138:A140"/>
+    <mergeCell ref="B138:B140"/>
+    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="C4:E5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="C7:E9"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="A35:A40"/>
+    <mergeCell ref="B35:B40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B54"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F146:F149"/>
   </mergeCells>
   <conditionalFormatting sqref="E10:E11 E2 E13:E58 E60:E70 E72:E78 E80:E81 E90:E93 E95:E115 E117:E122 E124:E140 E142:E149">
     <cfRule type="colorScale" priority="1">

</xml_diff>